<commit_message>
fix: 前十大投资信息bug修复 add by huzhangshun 2022/11/18
</commit_message>
<xml_diff>
--- a/tams-disclosure-parent/tams-disclosure/src/main/resources/tpl/InvestmentInfo.xlsx
+++ b/tams-disclosure-parent/tams-disclosure/src/main/resources/tpl/InvestmentInfo.xlsx
@@ -16,7 +16,7 @@
     <sheet name="接口数据要求" sheetId="3" r:id="rId2"/>
     <sheet name="报表影响点" sheetId="2" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
   <si>
     <t>持有份额</t>
   </si>
@@ -110,11 +110,25 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>产品名称*</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>持有份额*</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>占总份额比例*</t>
+  </si>
+  <si>
+    <t>数据状态*</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>更新时间*</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>更新人*</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -176,7 +190,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -192,6 +206,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -236,15 +256,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -277,6 +294,19 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -316,7 +346,7 @@
         <xdr:cNvPr id="2" name="图片 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{4546FE02-E43C-CE54-6251-41CE5B80DD19}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4546FE02-E43C-CE54-6251-41CE5B80DD19}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -608,42 +638,55 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.375" customWidth="1"/>
     <col min="2" max="2" width="11.5" customWidth="1"/>
     <col min="3" max="3" width="14.75" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="20.25" customWidth="1"/>
-    <col min="6" max="6" width="20.625" customWidth="1"/>
-    <col min="7" max="7" width="23" customWidth="1"/>
+    <col min="4" max="5" width="16" customWidth="1"/>
+    <col min="6" max="9" width="20.25" customWidth="1"/>
+    <col min="10" max="10" width="20.625" customWidth="1"/>
+    <col min="11" max="12" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:12" s="15" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>21</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L1" s="16"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -651,8 +694,13 @@
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="17"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -660,8 +708,13 @@
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="17"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -669,8 +722,13 @@
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="17"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -678,8 +736,13 @@
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="17"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -687,8 +750,13 @@
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="17"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -696,6 +764,11 @@
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="17"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -722,77 +795,77 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="13" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="15"/>
+      <c r="B3" s="14"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="15"/>
+      <c r="B4" s="14"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="15"/>
+      <c r="B5" s="14"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B6" s="5"/>
+      <c r="B6" s="4"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B7" s="5"/>
+      <c r="B7" s="4"/>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B8" s="5"/>
+      <c r="B8" s="4"/>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="5" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="11" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="11" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="5" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="B13" s="12" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>